<commit_message>
modif structure : un seul venv à la racine
</commit_message>
<xml_diff>
--- a/Lab/outils/work/normalized.xlsx
+++ b/Lab/outils/work/normalized.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J43"/>
+  <dimension ref="A1:J50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -483,7 +483,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -493,7 +493,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Les échos du passé</t>
+          <t>Urchin</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -504,98 +504,98 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Mascha Schilinski</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Prix du jury Cannes 2025</t>
-        </is>
-      </c>
+          <t>Harris Dickinson</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Découverte</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
+          <t>Grand Prix Jury de jeunes Carbonne fait son cinéma - Meilleure interprétation Un certain regard Cannes</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Coup de cœur</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Christy and his brother</t>
+          <t>Le sommet des dieux</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>VO</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>CM1</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Brendan Canty</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+          <t>VF</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2.8</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Coip de cœur</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
+          <t>Patrick Imbert</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>SCOL CauC</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Ma frère</t>
+          <t>Rue Malaga</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>VF</t>
+          <t>VO</t>
         </is>
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Lise Akoka, Romane Gueret</t>
+          <t>Maryam Touzani</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Séance EPHAD HANDI - Famille</t>
+          <t>Prix du public Venise</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Tarif Unique 5 €</t>
+          <t>Coup de cœur</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
@@ -603,53 +603,57 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Hamnet</t>
+          <t>Microcosmos</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>VO</t>
+          <t>VF</t>
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Chloé Zhao</t>
+          <t>Claude Nuridsany, Marie Pérennou</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Meilleure film dramatique et meilleure actrice Golden Globes 2026</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>SCOL EauC</t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Olivia</t>
+          <t>Alter ego</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -660,18 +664,18 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Irene Iborra</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Jeune Public</t>
-        </is>
-      </c>
+          <t>Nicolas Charlet, Bruno Lavaine</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>TU 5 €</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Tarif Unique 4,50 €</t>
+          <t>Séance EPHAD HANDI</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
@@ -679,39 +683,39 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Bardot</t>
+          <t>La couleuvre noire</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>VF</t>
+          <t>VO</t>
         </is>
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Alain Berliner, Elora Thevenet</t>
+          <t>Aurélien Vernhes-Lermusiaux</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Ciné Documentaire du samedi 18h</t>
+          <t>Prix Fondation Gan</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Adhérents 4 € - Autres 5 €</t>
+          <t>Cinélatino Avant-première</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
@@ -719,17 +723,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Grand ciel</t>
+          <t>L'ourse et l'oiseau</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -740,28 +744,36 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Akihiro Hata</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
+          <t>Marie Caudry, Aurore Peuffier, Nina Bisyarina</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>TU 3 €</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Jeune Public</t>
+        </is>
+      </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Biscuit le chien fantastique</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -772,64 +784,80 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Shea Wageman</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
+          <t>Edouard Bergeon</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>ADH 4 € - Autres 5 €</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Jeune Public</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr"/>
+          <t>invité Jérôme Bayle attente de réponse</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Ciné Documentaire du samedi 18h</t>
+        </is>
+      </c>
       <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>L'affaire Bojarski</t>
+          <t>Marty Supreme</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>VF</t>
+          <t>VO</t>
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Jean-Paul Salomé</t>
+          <t>Josh Safdie</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Golden Globe meilleur acteur</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Coup de cœur</t>
+        </is>
+      </c>
       <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Tafiti</t>
+          <t>Marsupilami</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -840,7 +868,7 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Nina Wels</t>
+          <t>Philippe Lacheau</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
@@ -849,95 +877,99 @@
           <t>Jeune Public</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Famille</t>
+        </is>
+      </c>
       <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Le mage du Kremlin</t>
+          <t>Maigret et le mort amoureux</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>VO</t>
+          <t>VF</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Olivier Assayas</t>
+          <t>Pascal Bonitzer</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Découverte</t>
-        </is>
-      </c>
+      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>The mastermind</t>
+          <t>Les Tourouges et les Toubleus</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>VO</t>
+          <t>VF</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Kelly Reichardt</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Découverte</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr"/>
+          <t>Samantha Cutler, Daniel Snaddon</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>SCOL Liste</t>
+        </is>
+      </c>
       <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Avatar De cendres et de feu</t>
+          <t>Coutures</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -948,22 +980,18 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>James Cameron</t>
+          <t>Alice Winocour</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Famille - 2D</t>
-        </is>
-      </c>
+      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -973,37 +1001,33 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>En garde</t>
+          <t>Pédale rurale</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>VO</t>
+          <t>VF</t>
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Nelicia Low</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Grand Prix du Jury La Roche sur Yon - Meilleur réalisation Karlovy Vary</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Découverte</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr"/>
+          <t>Antine Vasquez</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>DOC Découverte</t>
+        </is>
+      </c>
       <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1013,7 +1037,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Le gâteau du président</t>
+          <t>Little trouble girls</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1021,61 +1045,57 @@
           <t>VO</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>CM2</t>
-        </is>
-      </c>
+      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Hasan Hadi</t>
+          <t>Urška Djukić</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Coup de cœur</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Découverte</t>
+        </is>
+      </c>
       <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Les toutes petites créatures 2</t>
+          <t>Marty Supreme</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>VF</t>
+          <t>VO</t>
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Lucy Izzard</t>
+          <t>Josh Safdie</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Jeune Public</t>
+          <t>Golden Globe meilleur acteur</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Tarif Unique 3 €</t>
+          <t>Coup de cœur</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
@@ -1083,97 +1103,97 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Nuages flottants</t>
+          <t>Esprit(s) rebelle(s)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>VO</t>
+          <t>VF</t>
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Mikio Naruse</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr"/>
+          <t>Natalia Chernysheva</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>TU 3 €</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Ciné Patrimoine du samedi 18h</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>Adhérents 4 € - Autres 5 €</t>
-        </is>
-      </c>
+          <t>Jeune Public</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Palestine 36</t>
+          <t>Une balle dans la tête</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>VF</t>
+          <t>VO</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Annemarie Jacir</t>
+          <t>John Woo</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Grand Prix Tokyo - Meilleur film Milan</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>Coup de cœur</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr"/>
+          <t>ADH 4 € - Autres 5 €</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Ciné Patrimoine du samedi 18h</t>
+        </is>
+      </c>
       <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Le chant des forêts</t>
+          <t>Le rêve américain</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1184,36 +1204,28 @@
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Vincent Munier</t>
+          <t>Anthony Marciano</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>Documentaire Famille</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>Tarif Unique 4,50 €</t>
-        </is>
-      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Gourou</t>
+          <t>Le chant des forêts</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1224,18 +1236,22 @@
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Yann Gozlan</t>
+          <t>Vincent Munier</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>DOC Coup de coeur</t>
+        </is>
+      </c>
       <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1245,7 +1261,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Les légendaires</t>
+          <t>Les enfants de la Résistance</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1256,7 +1272,7 @@
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Guillaume Ivernel</t>
+          <t>Christophe Barratier</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -1265,23 +1281,27 @@
           <t>Jeune Public</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Famille</t>
+        </is>
+      </c>
       <c r="J22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Soulèvements</t>
+          <t>Chers parents</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1292,68 +1312,68 @@
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Thomas Lacoste</t>
+          <t>Emmanuel Patron</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>Documentaire</t>
-        </is>
-      </c>
+      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Les dimanches</t>
+          <t>Les enfants de la Résistance</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>VO</t>
+          <t>VF</t>
         </is>
       </c>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Alauda Ruíz de Azúa</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>Découverte</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr"/>
+          <t>Christophe Barratier</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>SCOL Actu</t>
+        </is>
+      </c>
       <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Les toutes petites créatures 2</t>
+          <t>Victor comme tout le monde</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1364,26 +1384,18 @@
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Lucy Izzard</t>
+          <t>Pascal Bonitzer</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>Jeune Public</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>Tarif Unique 3 €</t>
-        </is>
-      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1393,7 +1405,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Nurenberg</t>
+          <t>La gifle</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1404,54 +1416,50 @@
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
-          <t>James Vanderbilt</t>
+          <t>Frédéric Hambalek</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr">
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
         <is>
           <t>Découverte</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Marsupilami JP famille</t>
+          <t>Ce qu'il reste de nous</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>VF</t>
+          <t>VO</t>
         </is>
       </c>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Philippe Lacheau</t>
+          <t>Cherien Dabis</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>Séance EPHAD HANDI - Famille</t>
-        </is>
-      </c>
+      <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Tarif Unique 5 €</t>
+          <t>Découverte</t>
         </is>
       </c>
       <c r="J27" t="inlineStr"/>
@@ -1459,75 +1467,75 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Aucun autre choix</t>
+          <t>Le rêve américain</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>VO</t>
+          <t>VF</t>
         </is>
       </c>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Park Chan-Wook</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>Coup de cœur</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr"/>
+          <t>Anthony Marciano</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>TU 5 €</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Séance EPHAD HANDI</t>
+        </is>
+      </c>
       <c r="J28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Biscuit le chien fantastique</t>
+          <t>Un monde fragile et merveilleux</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>VF</t>
+          <t>VO</t>
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Shea Wageman</t>
+          <t>Cyril Aris</t>
         </is>
       </c>
       <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>Ciné goûter, Jeune Public</t>
-        </is>
-      </c>
+      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Tarif Unique 4,50 €</t>
+          <t>Coup de cœur</t>
         </is>
       </c>
       <c r="J29" t="inlineStr"/>
@@ -1535,43 +1543,43 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Hamnet</t>
+          <t>Jumpers</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>VO</t>
+          <t>VF</t>
         </is>
       </c>
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Chloé Zhao</t>
+          <t>Daniel Chong</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Meilleure film dramatique et meilleure actrice Golden Globes 2026</t>
+          <t>TU 4,50 €</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Ciné Jeunes du samedi 18h</t>
+          <t>Jeune Public</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Adhérents 4 € - Autres 5 €</t>
+          <t>Ciné goûter</t>
         </is>
       </c>
       <c r="J30" t="inlineStr"/>
@@ -1579,49 +1587,57 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>A pied d'œuvre</t>
+          <t>Christy</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>VF</t>
+          <t>VO</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Valérie Donzelli</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr"/>
+          <t>David Michôd</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>ADH 4 € - Autres 5 €</t>
+        </is>
+      </c>
       <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Ciné Jeunes du samedi 18h</t>
+        </is>
+      </c>
       <c r="J31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Les légendaires</t>
+          <t>La maison des femmes</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1632,32 +1648,28 @@
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Guillaume Ivernel</t>
+          <t>Melisa Godet</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>Jeune Public</t>
-        </is>
-      </c>
+      <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Promis le ciel</t>
+          <t>Allah n'est pas obligé</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1668,32 +1680,36 @@
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Erige Sehiri</t>
+          <t>Zaven Najjar</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Coup de cœur</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr"/>
+          <t>Jeune Public</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Famille  à partir de 9/10 ans</t>
+        </is>
+      </c>
       <c r="J33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Gourou</t>
+          <t>La guerre des prix</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1704,7 +1720,7 @@
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Yann Gozlan</t>
+          <t>Anthony Dechaux</t>
         </is>
       </c>
       <c r="G34" t="inlineStr"/>
@@ -1715,7 +1731,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1725,83 +1741,71 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Les voyages de Tereza</t>
+          <t>Alter ego</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>VO</t>
+          <t>VF</t>
         </is>
       </c>
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Gabriel Mascaro</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>Cinélatino</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>Coup de cœur</t>
-        </is>
-      </c>
+          <t>Nicolas Charlet, Bruno Lavaine</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Dreams</t>
+          <t>Le rêve américain</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>VO</t>
+          <t>VF</t>
         </is>
       </c>
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Michel Franco</t>
+          <t>Anthony Marciano</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>Découverte</t>
-        </is>
-      </c>
+      <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Lol 2.0</t>
+          <t>Les figures de l'ombre</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1812,64 +1816,72 @@
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Lisa Azuelos</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr"/>
+          <t>Theodore Melfi</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>SCOL Pass culture</t>
+        </is>
+      </c>
       <c r="J37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Super Charlie</t>
+          <t>Woman and child VO</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>VF</t>
+          <t>VO</t>
         </is>
       </c>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Jon Holmberg</t>
+          <t>Saeed Roustaee</t>
         </is>
       </c>
       <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>Jeune Public</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Découverte</t>
+        </is>
+      </c>
       <c r="J38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Abel</t>
+          <t>Pillion</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1880,22 +1892,14 @@
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Elzat Eskendir</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>Grand Prix et Prix de la critique Vesoul 2025</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>Ciné discussion - Coup ce cœur</t>
-        </is>
-      </c>
+          <t>Harry Lighton</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Adhérents 4 € - Autres 5 €</t>
+          <t>Découverte</t>
         </is>
       </c>
       <c r="J39" t="inlineStr"/>
@@ -1903,17 +1907,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Maigret et le mort amoureux</t>
+          <t>Le chant de la mer</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1924,50 +1928,54 @@
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Pascal Bonitzer</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr"/>
+          <t>Tomm Moore</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>SCOL liste</t>
+        </is>
+      </c>
       <c r="J40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Tafiti</t>
+          <t>Love on trial</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>VF</t>
+          <t>VO</t>
         </is>
       </c>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Nina Wels</t>
+          <t>Kôji Fukada</t>
         </is>
       </c>
       <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>Jeune Public</t>
-        </is>
-      </c>
+      <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Tarif Unique 4,50 €</t>
+          <t>Découverte</t>
         </is>
       </c>
       <c r="J41" t="inlineStr"/>
@@ -1975,78 +1983,342 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Les enfants de la Résistance</t>
+          <t>Il maestro</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>VF</t>
+          <t>VO</t>
         </is>
       </c>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Christophe Barratier</t>
+          <t>Andrea di Stefano</t>
         </is>
       </c>
       <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>Famille, Jeune Public</t>
-        </is>
-      </c>
+      <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Le mystérieux regard du flamant rose</t>
+          <t>Scarlet et l'éternité</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>VO</t>
+          <t>VF</t>
         </is>
       </c>
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Diego Cespedes</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>Cinélatino</t>
-        </is>
-      </c>
+          <t>Mamoru Hosoda</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
+          <t>Jeune Public</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>ados à partir de 9/10 ans Sony</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>La grazia</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>VO</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Paolo Sorrentino</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>ADH 4 € - Autres 5 €</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Ciné Discussion du samedi 18h</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Le son des souvenirs</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>VO</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Oliver Hermanus</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr">
+        <is>
           <t>Coup de cœur</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Planètes</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>VF</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Momoko Seto</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>TU 4,50 €</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Jeune Public</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Famille</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Le crime du 3e étage</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>VF</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Rémi Bezançon</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Léo la fabuleuse histoire de Léonard de Vinci</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>VF</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Jim Capobianco</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>3.8</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>SCOL EauC</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Léo la fabuleuse histoire de Léonard de Vinci</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>VF</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Jim Capobianco</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>3.8</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>SCOL EauC</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Les filles du ciel</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>VF</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Bérangère Mc Neese</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Découverte</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>